<commit_message>
1eres simulations débits CV1 (scenario 1)
Résultats des premières simulations de débits potentiellement récupérable dans la CV1 lors du recoupement de conduits karstiques pendant l'excavation. Les simulations sont données pour T3, T10, T30 et T50, aprés la phase 1.8a d'excavation du Twanntunnel.
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882AFE1A-18AF-4F60-9FDC-3D4CBD85339A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A11C5CA-95B3-4FB7-A32B-1ACCB278A640}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20235" windowHeight="9060" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="64">
   <si>
     <t>Holiloch_sonde</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>TWT_PointHaut_60+749</t>
+  </si>
+  <si>
+    <t>CentraleVentilation_1C</t>
   </si>
 </sst>
 </file>
@@ -586,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336D857F-22C8-4624-8585-90FCE8727574}">
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1808,6 +1811,22 @@
         <v>348</v>
       </c>
     </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B84" s="3">
+        <v>2578077</v>
+      </c>
+      <c r="C84" s="3">
+        <v>1215700</v>
+      </c>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3">
+        <v>454</v>
+      </c>
+      <c r="F84" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>